<commit_message>
Solved hyperarcid and designlines
</commit_message>
<xml_diff>
--- a/test/configs/data/develop/multilink.xlsx
+++ b/test/configs/data/develop/multilink.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="7824" activeTab="3"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="7824" activeTab="5"/>
   </bookViews>
   <sheets>
     <sheet name="Carrier" sheetId="4" r:id="rId1"/>
@@ -31,7 +31,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="124" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="72">
   <si>
     <t>solar</t>
   </si>
@@ -220,6 +220,33 @@
   </si>
   <si>
     <t>line 0-1</t>
+  </si>
+  <si>
+    <t>bus 3</t>
+  </si>
+  <si>
+    <t>demand 3</t>
+  </si>
+  <si>
+    <t>bus3</t>
+  </si>
+  <si>
+    <t>efficiency3</t>
+  </si>
+  <si>
+    <t>bus 4</t>
+  </si>
+  <si>
+    <t>demand 4</t>
+  </si>
+  <si>
+    <t>bus4</t>
+  </si>
+  <si>
+    <t>efficiency4</t>
+  </si>
+  <si>
+    <t>batterylink 2</t>
   </si>
 </sst>
 </file>
@@ -665,7 +692,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:G4"/>
+  <dimension ref="A1:G6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="7" width="8.88671875" style="1"/>
@@ -739,6 +766,40 @@
         <v>0.4</v>
       </c>
     </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1">
+        <v>6</v>
+      </c>
+      <c r="D5" s="1">
+        <v>0</v>
+      </c>
+      <c r="E5" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1">
+        <v>8</v>
+      </c>
+      <c r="D6" s="1">
+        <v>0</v>
+      </c>
+      <c r="E6" s="1">
+        <v>0.4</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -746,7 +807,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:E6"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="5" width="8.88671875" style="1"/>
@@ -794,6 +855,28 @@
       </c>
       <c r="C4" s="1" t="s">
         <v>54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A5" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="B5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>63</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A6" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="B6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>67</v>
       </c>
     </row>
   </sheetData>
@@ -988,7 +1071,7 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:M3"/>
+  <dimension ref="A1:Q4"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="10.109375" bestFit="1" customWidth="1"/>
@@ -997,7 +1080,7 @@
     <col min="7" max="7" width="9.44140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1037,8 +1120,20 @@
       <c r="M1" s="1" t="s">
         <v>61</v>
       </c>
-    </row>
-    <row r="2" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="N1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="P1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="2" spans="1:17" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>59</v>
       </c>
@@ -1075,7 +1170,7 @@
         <v>0.01</v>
       </c>
     </row>
-    <row r="3" spans="1:13" s="1" customFormat="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>56</v>
       </c>
@@ -1098,7 +1193,7 @@
         <v>1</v>
       </c>
       <c r="H3" s="1">
-        <v>0.5</v>
+        <v>0.4</v>
       </c>
       <c r="I3" s="1">
         <v>10</v>
@@ -1107,13 +1202,78 @@
         <v>54</v>
       </c>
       <c r="K3" s="1">
-        <v>0.4</v>
+        <v>0.3</v>
       </c>
       <c r="L3" s="1">
         <v>60</v>
       </c>
       <c r="M3" s="1">
         <v>0.01</v>
+      </c>
+      <c r="N3" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="O3" s="1">
+        <v>0.2</v>
+      </c>
+      <c r="P3" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q3" s="1">
+        <v>0.1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:17" s="1" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="F4" s="1">
+        <v>0</v>
+      </c>
+      <c r="G4" s="1">
+        <v>1</v>
+      </c>
+      <c r="H4" s="1">
+        <v>0.3</v>
+      </c>
+      <c r="I4" s="1">
+        <v>0</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>54</v>
+      </c>
+      <c r="K4" s="1">
+        <v>0.05</v>
+      </c>
+      <c r="L4" s="1">
+        <v>70</v>
+      </c>
+      <c r="M4" s="1">
+        <v>0.02</v>
+      </c>
+      <c r="N4" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="O4" s="1">
+        <v>0.15</v>
+      </c>
+      <c r="P4" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="Q4" s="1">
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>